<commit_message>
feat: complete Phase 8 (Retest) and Phase 9 (Regression Testing with 100% PASS)
</commit_message>
<xml_diff>
--- a/3. DefectReport.xlsx
+++ b/3. DefectReport.xlsx
@@ -1685,12 +1685,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Chay on dinh</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1727,12 +1727,12 @@
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H3" s="9" t="inlineStr">
         <is>
-          <t>Xu ly an toan</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1769,12 +1769,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Bao mat tot</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1811,12 +1811,12 @@
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>Client validation</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1853,12 +1853,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Boundary OK</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1895,12 +1895,12 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>Trang hoat dong tot</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1937,12 +1937,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Validation form dung</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -1979,12 +1979,12 @@
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>Khong bi anh huong</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -2021,12 +2021,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Bao mat OK</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>
@@ -2063,12 +2063,12 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-10-04 22:14:55</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>Core page OK</t>
+          <t>Xac minh chay thuc te qua Maven: 100% PASS</t>
         </is>
       </c>
     </row>

</xml_diff>